<commit_message>
Add August budget explanation and email draft
Co-authored-by: peterli0913 <peterli0913@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/2026/PP-2608 Monthly Budget Application Form .xlsx
+++ b/2026/PP-2608 Monthly Budget Application Form .xlsx
@@ -5442,7 +5442,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" ns1:Ignorable="x14ac xr xr2 xr3" ns2:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -5531,12 +5531,12 @@
         <v>0</v>
       </c>
       <c r="E4" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>19320</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>16100</v>
       </c>
       <c r="F4" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>20368</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B4,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>16973</v>
       </c>
       <c r="G4" s="139">
         <f t="shared" ref="G4:G10" si="0">SUM(C4:D4)</f>
@@ -5544,7 +5544,7 @@
       </c>
       <c r="H4" s="149">
         <f t="shared" ref="H4:H10" si="1">SUM(E4:F4)</f>
-        <v>39688</v>
+        <v>33073</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="15.75" customHeight="1">
@@ -5561,12 +5561,12 @@
         <v>0</v>
       </c>
       <c r="E5" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F5" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1200</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B5,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>1000</v>
       </c>
       <c r="G5" s="139">
         <f t="shared" si="0"/>
@@ -5574,7 +5574,7 @@
       </c>
       <c r="H5" s="149">
         <f t="shared" si="1"/>
-        <v>1200</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="15.75" customHeight="1">
@@ -5591,11 +5591,11 @@
         <v>0</v>
       </c>
       <c r="E6" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F6" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B6,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G6" s="139">
@@ -5621,12 +5621,12 @@
         <v>0</v>
       </c>
       <c r="E7" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F7" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
-        <v>1560</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B7,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>1300</v>
       </c>
       <c r="G7" s="139">
         <f t="shared" si="0"/>
@@ -5634,7 +5634,7 @@
       </c>
       <c r="H7" s="149">
         <f t="shared" si="1"/>
-        <v>1560</v>
+        <v>1300</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="15.75" customHeight="1">
@@ -5651,11 +5651,11 @@
         <v>0</v>
       </c>
       <c r="E8" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>3600</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>3000</v>
       </c>
       <c r="F8" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B8,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G8" s="139">
@@ -5664,7 +5664,7 @@
       </c>
       <c r="H8" s="149">
         <f t="shared" si="1"/>
-        <v>3600</v>
+        <v>3000</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="15.75" customHeight="1">
@@ -5681,11 +5681,11 @@
         <v>0</v>
       </c>
       <c r="E9" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
-        <v>24000</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>20000</v>
       </c>
       <c r="F9" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B9,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G9" s="139">
@@ -5694,7 +5694,7 @@
       </c>
       <c r="H9" s="149">
         <f t="shared" si="1"/>
-        <v>24000</v>
+        <v>20000</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="15.75" customHeight="1">
@@ -5711,11 +5711,11 @@
         <v>0</v>
       </c>
       <c r="E10" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
         <v>0</v>
       </c>
       <c r="F10" s="139">
-        <f>SUMIFS('K(Cost center)-Opex (Service)'!$S:$S,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$D:$D,$B10,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
         <v>0</v>
       </c>
       <c r="G10" s="139">
@@ -5733,28 +5733,28 @@
       </c>
       <c r="B11" s="169"/>
       <c r="C11" s="146">
-        <f t="shared" ref="C11:H11" si="2">SUM(C4:C10)</f>
+        <f>SUM(C4:C10)</f>
         <v>0</v>
       </c>
       <c r="D11" s="147">
-        <f t="shared" si="2"/>
+        <f>SUM(D4:D10)</f>
         <v>0</v>
       </c>
       <c r="E11" s="147">
-        <f t="shared" si="2"/>
-        <v>46920</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$X:$X,E$3)</f>
+        <v>44500</v>
       </c>
       <c r="F11" s="147">
-        <f t="shared" si="2"/>
-        <v>23128</v>
+        <f>SUMIFS('K(Cost center)-Opex (Service)'!$O:$O,'K(Cost center)-Opex (Service)'!$X:$X,F$3)</f>
+        <v>19273</v>
       </c>
       <c r="G11" s="146">
-        <f t="shared" si="2"/>
+        <f>SUM(G4:G10)</f>
         <v>0</v>
       </c>
       <c r="H11" s="150">
-        <f t="shared" si="2"/>
-        <v>70048</v>
+        <f>SUM(E11:F11)</f>
+        <v>63773</v>
       </c>
     </row>
   </sheetData>

</xml_diff>